<commit_message>
;- gea f83hxq2.z le82gew2
</commit_message>
<xml_diff>
--- a/MyWebExercise_02App/wwwroot/template/my_template.xlsx
+++ b/MyWebExercise_02App/wwwroot/template/my_template.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="26">
   <si>
     <t xml:space="preserve">系統名稱</t>
   </si>
@@ -51,6 +51,9 @@
   </si>
   <si>
     <t xml:space="preserve">#table.description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">返回清單</t>
   </si>
   <si>
     <t xml:space="preserve">資料表描述</t>
@@ -105,7 +108,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <sz val="10"/>
       <name val="Noto Sans TC"/>
@@ -152,6 +155,22 @@
     <font>
       <sz val="10"/>
       <name val="微軟正黑體"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <u val="single"/>
+      <sz val="14"/>
+      <color theme="10"/>
+      <name val="微軟正黑體"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <u val="single"/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
@@ -164,7 +183,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -186,8 +205,22 @@
       <bottom style="thin"/>
       <diagonal/>
     </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="20">
+  <cellStyleXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -211,8 +244,11 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -249,18 +285,31 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="7">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Comma" xfId="15" builtinId="3"/>
     <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
     <cellStyle name="Currency" xfId="17" builtinId="4"/>
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
+    <cellStyle name="*unknown*" xfId="20" builtinId="8"/>
   </cellStyles>
 </styleSheet>
 </file>
@@ -517,7 +566,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultColWidth="3.42578125" defaultRowHeight="24.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="8" width="7.71"/>
@@ -528,6 +577,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="8" width="20.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="8" width="20.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="8" width="41.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="9" width="10.89"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -535,18 +585,20 @@
         <v>5</v>
       </c>
       <c r="B1" s="2"/>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="11" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2" t="s">
@@ -557,28 +609,29 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
+      <c r="I2" s="0"/>
     </row>
     <row r="3" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H3" s="6" t="s">
         <v>6</v>
@@ -586,37 +639,40 @@
     </row>
     <row r="4" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="C4" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="D4" s="12" t="s">
         <v>21</v>
       </c>
+      <c r="E4" s="12" t="s">
+        <v>22</v>
+      </c>
       <c r="F4" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:H1"/>
+    <mergeCell ref="C1:G1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:H2"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="H1" location="'Table List'!A1" display="返回清單"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>